<commit_message>
feat: add comprehensive 10-site microbial encyclopedia, exact DNA NGS profiles, and stand filters
</commit_message>
<xml_diff>
--- a/aerobiome_analysis_summary.xlsx
+++ b/aerobiome_analysis_summary.xlsx
@@ -22,6 +22,7 @@
     <sheet name="6Dates_Site_TAB_Matrix" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="6Dates_Environmental_Corr" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="6Dates_IAQ_Compliance" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Site_Microbial_Encyclopedia" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2148,7 +2149,6 @@
       <c r="Q2" t="n">
         <v>48</v>
       </c>
-      <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr">
         <is>
           <t>리기다소나무림</t>
@@ -2272,7 +2272,6 @@
       <c r="Q3" t="n">
         <v>26</v>
       </c>
-      <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr">
         <is>
           <t>리기다소나무림</t>
@@ -2396,7 +2395,6 @@
       <c r="Q4" t="n">
         <v>31</v>
       </c>
-      <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr">
         <is>
           <t>리기다소나무림</t>
@@ -2520,7 +2518,6 @@
       <c r="Q5" t="n">
         <v>31</v>
       </c>
-      <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr">
         <is>
           <t>리기다소나무림</t>
@@ -2644,7 +2641,6 @@
       <c r="Q6" t="n">
         <v>31</v>
       </c>
-      <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr">
         <is>
           <t>리기다소나무림</t>
@@ -2768,7 +2764,6 @@
       <c r="Q7" t="n">
         <v>15</v>
       </c>
-      <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr">
         <is>
           <t>잣나무림 a</t>
@@ -2892,7 +2887,6 @@
       <c r="Q8" t="n">
         <v>46</v>
       </c>
-      <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr">
         <is>
           <t>잣나무림 a</t>
@@ -3016,7 +3010,6 @@
       <c r="Q9" t="n">
         <v>15</v>
       </c>
-      <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr">
         <is>
           <t>잣나무림 a</t>
@@ -3140,7 +3133,6 @@
       <c r="Q10" t="n">
         <v>15</v>
       </c>
-      <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr">
         <is>
           <t>잣나무림 a</t>
@@ -3264,7 +3256,6 @@
       <c r="Q11" t="n">
         <v>15</v>
       </c>
-      <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr">
         <is>
           <t>잣나무림 a</t>
@@ -3388,7 +3379,6 @@
       <c r="Q12" t="n">
         <v>175</v>
       </c>
-      <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr">
         <is>
           <t>버들나무림 a</t>
@@ -3512,7 +3502,6 @@
       <c r="Q13" t="n">
         <v>26</v>
       </c>
-      <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr">
         <is>
           <t>버들나무림 a</t>
@@ -3636,7 +3625,6 @@
       <c r="Q14" t="n">
         <v>68</v>
       </c>
-      <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr">
         <is>
           <t>버들나무림 a</t>
@@ -3760,7 +3748,6 @@
       <c r="Q15" t="n">
         <v>33</v>
       </c>
-      <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr">
         <is>
           <t>버들나무림 a</t>
@@ -3884,7 +3871,6 @@
       <c r="Q16" t="n">
         <v>50.5</v>
       </c>
-      <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr">
         <is>
           <t>버들나무림 a</t>
@@ -4008,7 +3994,6 @@
       <c r="Q17" t="n">
         <v>9</v>
       </c>
-      <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr">
         <is>
           <t>밭(대조구)</t>
@@ -4132,7 +4117,6 @@
       <c r="Q18" t="n">
         <v>9</v>
       </c>
-      <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr">
         <is>
           <t>밭(대조구)</t>
@@ -4256,7 +4240,6 @@
       <c r="Q19" t="n">
         <v>7</v>
       </c>
-      <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr">
         <is>
           <t>밭(대조구)</t>
@@ -4380,7 +4363,6 @@
       <c r="Q20" t="n">
         <v>9</v>
       </c>
-      <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr">
         <is>
           <t>밭(대조구)</t>
@@ -4504,7 +4486,6 @@
       <c r="Q21" t="n">
         <v>9</v>
       </c>
-      <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr">
         <is>
           <t>밭(대조구)</t>
@@ -4628,7 +4609,6 @@
       <c r="Q22" t="n">
         <v>3</v>
       </c>
-      <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr">
         <is>
           <t>주차장(대조구)</t>
@@ -4752,7 +4732,6 @@
       <c r="Q23" t="n">
         <v>5</v>
       </c>
-      <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr">
         <is>
           <t>주차장(대조구)</t>
@@ -4876,7 +4855,6 @@
       <c r="Q24" t="n">
         <v>8</v>
       </c>
-      <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr">
         <is>
           <t>주차장(대조구)</t>
@@ -5000,7 +4978,6 @@
       <c r="Q25" t="n">
         <v>13</v>
       </c>
-      <c r="R25" t="inlineStr"/>
       <c r="S25" t="inlineStr">
         <is>
           <t>소나무림</t>
@@ -5124,7 +5101,6 @@
       <c r="Q26" t="n">
         <v>18</v>
       </c>
-      <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr">
         <is>
           <t>소나무림</t>
@@ -5248,7 +5224,6 @@
       <c r="Q27" t="n">
         <v>15</v>
       </c>
-      <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr">
         <is>
           <t>소나무림</t>
@@ -5372,7 +5347,6 @@
       <c r="Q28" t="n">
         <v>18</v>
       </c>
-      <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr">
         <is>
           <t>소나무림</t>
@@ -5496,7 +5470,6 @@
       <c r="Q29" t="n">
         <v>27</v>
       </c>
-      <c r="R29" t="inlineStr"/>
       <c r="S29" t="inlineStr">
         <is>
           <t>소나무림</t>
@@ -5620,7 +5593,6 @@
       <c r="Q30" t="n">
         <v>47</v>
       </c>
-      <c r="R30" t="inlineStr"/>
       <c r="S30" t="inlineStr">
         <is>
           <t>일본잎갈나무림 a</t>
@@ -5744,7 +5716,6 @@
       <c r="Q31" t="n">
         <v>15</v>
       </c>
-      <c r="R31" t="inlineStr"/>
       <c r="S31" t="inlineStr">
         <is>
           <t>일본잎갈나무림 a</t>
@@ -5868,7 +5839,6 @@
       <c r="Q32" t="n">
         <v>21</v>
       </c>
-      <c r="R32" t="inlineStr"/>
       <c r="S32" t="inlineStr">
         <is>
           <t>일본잎갈나무림 a</t>
@@ -5992,7 +5962,6 @@
       <c r="Q33" t="n">
         <v>16</v>
       </c>
-      <c r="R33" t="inlineStr"/>
       <c r="S33" t="inlineStr">
         <is>
           <t>일본잎갈나무림 a</t>
@@ -6116,7 +6085,6 @@
       <c r="Q34" t="n">
         <v>50</v>
       </c>
-      <c r="R34" t="inlineStr"/>
       <c r="S34" t="inlineStr">
         <is>
           <t>일본잎갈나무림 a</t>
@@ -6240,7 +6208,6 @@
       <c r="Q35" t="n">
         <v>69</v>
       </c>
-      <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr">
         <is>
           <t>버들나무림 b</t>
@@ -6364,7 +6331,6 @@
       <c r="Q36" t="n">
         <v>132</v>
       </c>
-      <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr">
         <is>
           <t>버들나무림 b</t>
@@ -6488,7 +6454,6 @@
       <c r="Q37" t="n">
         <v>21</v>
       </c>
-      <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr">
         <is>
           <t>버들나무림 b</t>
@@ -6612,7 +6577,6 @@
       <c r="Q38" t="n">
         <v>37</v>
       </c>
-      <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr">
         <is>
           <t>버들나무림 b</t>
@@ -6736,7 +6700,6 @@
       <c r="Q39" t="n">
         <v>115</v>
       </c>
-      <c r="R39" t="inlineStr"/>
       <c r="S39" t="inlineStr">
         <is>
           <t>버들나무림 b</t>
@@ -6860,7 +6823,6 @@
       <c r="Q40" t="n">
         <v>79</v>
       </c>
-      <c r="R40" t="inlineStr"/>
       <c r="S40" t="inlineStr">
         <is>
           <t>일본잎갈나무림 b</t>
@@ -6984,7 +6946,6 @@
       <c r="Q41" t="n">
         <v>44</v>
       </c>
-      <c r="R41" t="inlineStr"/>
       <c r="S41" t="inlineStr">
         <is>
           <t>일본잎갈나무림 b</t>
@@ -7108,7 +7069,6 @@
       <c r="Q42" t="n">
         <v>33</v>
       </c>
-      <c r="R42" t="inlineStr"/>
       <c r="S42" t="inlineStr">
         <is>
           <t>일본잎갈나무림 b</t>
@@ -7232,7 +7192,6 @@
       <c r="Q43" t="n">
         <v>12</v>
       </c>
-      <c r="R43" t="inlineStr"/>
       <c r="S43" t="inlineStr">
         <is>
           <t>일본잎갈나무림 b</t>
@@ -7356,7 +7315,6 @@
       <c r="Q44" t="n">
         <v>23</v>
       </c>
-      <c r="R44" t="inlineStr"/>
       <c r="S44" t="inlineStr">
         <is>
           <t>일본잎갈나무림 b</t>
@@ -7480,7 +7438,6 @@
       <c r="Q45" t="n">
         <v>0</v>
       </c>
-      <c r="R45" t="inlineStr"/>
       <c r="S45" t="inlineStr">
         <is>
           <t>잣나무림 b</t>
@@ -7604,7 +7561,6 @@
       <c r="Q46" t="n">
         <v>32</v>
       </c>
-      <c r="R46" t="inlineStr"/>
       <c r="S46" t="inlineStr">
         <is>
           <t>잣나무림 b</t>
@@ -7728,7 +7684,6 @@
       <c r="Q47" t="n">
         <v>17</v>
       </c>
-      <c r="R47" t="inlineStr"/>
       <c r="S47" t="inlineStr">
         <is>
           <t>잣나무림 b</t>
@@ -7852,7 +7807,6 @@
       <c r="Q48" t="n">
         <v>26</v>
       </c>
-      <c r="R48" t="inlineStr"/>
       <c r="S48" t="inlineStr">
         <is>
           <t>잣나무림 b</t>
@@ -7976,7 +7930,6 @@
       <c r="Q49" t="n">
         <v>23</v>
       </c>
-      <c r="R49" t="inlineStr"/>
       <c r="S49" t="inlineStr">
         <is>
           <t>잣나무림 b</t>
@@ -8100,7 +8053,6 @@
       <c r="Q50" t="n">
         <v>41</v>
       </c>
-      <c r="R50" t="inlineStr"/>
       <c r="S50" t="inlineStr">
         <is>
           <t>리기다소나무림</t>
@@ -8224,7 +8176,6 @@
       <c r="Q51" t="n">
         <v>37</v>
       </c>
-      <c r="R51" t="inlineStr"/>
       <c r="S51" t="inlineStr">
         <is>
           <t>리기다소나무림</t>
@@ -8348,7 +8299,6 @@
       <c r="Q52" t="n">
         <v>42</v>
       </c>
-      <c r="R52" t="inlineStr"/>
       <c r="S52" t="inlineStr">
         <is>
           <t>리기다소나무림</t>
@@ -8472,7 +8422,6 @@
       <c r="Q53" t="n">
         <v>176</v>
       </c>
-      <c r="R53" t="inlineStr"/>
       <c r="S53" t="inlineStr">
         <is>
           <t>리기다소나무림</t>
@@ -8596,7 +8545,6 @@
       <c r="Q54" t="n">
         <v>48</v>
       </c>
-      <c r="R54" t="inlineStr"/>
       <c r="S54" t="inlineStr">
         <is>
           <t>리기다소나무림</t>
@@ -8720,7 +8668,6 @@
       <c r="Q55" t="n">
         <v>37</v>
       </c>
-      <c r="R55" t="inlineStr"/>
       <c r="S55" t="inlineStr">
         <is>
           <t>잣나무림 a</t>
@@ -8844,7 +8791,6 @@
       <c r="Q56" t="n">
         <v>144</v>
       </c>
-      <c r="R56" t="inlineStr"/>
       <c r="S56" t="inlineStr">
         <is>
           <t>잣나무림 a</t>
@@ -8968,7 +8914,6 @@
       <c r="Q57" t="n">
         <v>43</v>
       </c>
-      <c r="R57" t="inlineStr"/>
       <c r="S57" t="inlineStr">
         <is>
           <t>잣나무림 a</t>
@@ -9092,7 +9037,6 @@
       <c r="Q58" t="n">
         <v>95</v>
       </c>
-      <c r="R58" t="inlineStr"/>
       <c r="S58" t="inlineStr">
         <is>
           <t>잣나무림 a</t>
@@ -9216,7 +9160,6 @@
       <c r="Q59" t="n">
         <v>46</v>
       </c>
-      <c r="R59" t="inlineStr"/>
       <c r="S59" t="inlineStr">
         <is>
           <t>잣나무림 a</t>
@@ -9340,7 +9283,6 @@
       <c r="Q60" t="n">
         <v>56</v>
       </c>
-      <c r="R60" t="inlineStr"/>
       <c r="S60" t="inlineStr">
         <is>
           <t>버들나무림 a</t>
@@ -9464,7 +9406,6 @@
       <c r="Q61" t="n">
         <v>140</v>
       </c>
-      <c r="R61" t="inlineStr"/>
       <c r="S61" t="inlineStr">
         <is>
           <t>버들나무림 a</t>
@@ -9588,7 +9529,6 @@
       <c r="Q62" t="n">
         <v>54</v>
       </c>
-      <c r="R62" t="inlineStr"/>
       <c r="S62" t="inlineStr">
         <is>
           <t>버들나무림 a</t>
@@ -9712,7 +9652,6 @@
       <c r="Q63" t="n">
         <v>70</v>
       </c>
-      <c r="R63" t="inlineStr"/>
       <c r="S63" t="inlineStr">
         <is>
           <t>버들나무림 a</t>
@@ -9836,7 +9775,6 @@
       <c r="Q64" t="n">
         <v>47</v>
       </c>
-      <c r="R64" t="inlineStr"/>
       <c r="S64" t="inlineStr">
         <is>
           <t>버들나무림 a</t>
@@ -9960,7 +9898,6 @@
       <c r="Q65" t="n">
         <v>112</v>
       </c>
-      <c r="R65" t="inlineStr"/>
       <c r="S65" t="inlineStr">
         <is>
           <t>밭(대조구)</t>
@@ -10084,7 +10021,6 @@
       <c r="Q66" t="n">
         <v>183</v>
       </c>
-      <c r="R66" t="inlineStr"/>
       <c r="S66" t="inlineStr">
         <is>
           <t>밭(대조구)</t>
@@ -10208,7 +10144,6 @@
       <c r="Q67" t="n">
         <v>146</v>
       </c>
-      <c r="R67" t="inlineStr"/>
       <c r="S67" t="inlineStr">
         <is>
           <t>밭(대조구)</t>
@@ -10332,7 +10267,6 @@
       <c r="Q68" t="n">
         <v>95</v>
       </c>
-      <c r="R68" t="inlineStr"/>
       <c r="S68" t="inlineStr">
         <is>
           <t>밭(대조구)</t>
@@ -10456,7 +10390,6 @@
       <c r="Q69" t="n">
         <v>83</v>
       </c>
-      <c r="R69" t="inlineStr"/>
       <c r="S69" t="inlineStr">
         <is>
           <t>밭(대조구)</t>
@@ -10580,7 +10513,6 @@
       <c r="Q70" t="n">
         <v>49</v>
       </c>
-      <c r="R70" t="inlineStr"/>
       <c r="S70" t="inlineStr">
         <is>
           <t>주차장(대조구)</t>
@@ -10704,7 +10636,6 @@
       <c r="Q71" t="n">
         <v>44</v>
       </c>
-      <c r="R71" t="inlineStr"/>
       <c r="S71" t="inlineStr">
         <is>
           <t>주차장(대조구)</t>
@@ -10828,7 +10759,6 @@
       <c r="Q72" t="n">
         <v>66</v>
       </c>
-      <c r="R72" t="inlineStr"/>
       <c r="S72" t="inlineStr">
         <is>
           <t>주차장(대조구)</t>
@@ -10952,7 +10882,6 @@
       <c r="Q73" t="n">
         <v>32</v>
       </c>
-      <c r="R73" t="inlineStr"/>
       <c r="S73" t="inlineStr">
         <is>
           <t>주차장(대조구)</t>
@@ -11076,7 +11005,6 @@
       <c r="Q74" t="n">
         <v>37</v>
       </c>
-      <c r="R74" t="inlineStr"/>
       <c r="S74" t="inlineStr">
         <is>
           <t>주차장(대조구)</t>
@@ -11200,7 +11128,6 @@
       <c r="Q75" t="n">
         <v>38</v>
       </c>
-      <c r="R75" t="inlineStr"/>
       <c r="S75" t="inlineStr">
         <is>
           <t>소나무림</t>
@@ -11324,7 +11251,6 @@
       <c r="Q76" t="n">
         <v>33</v>
       </c>
-      <c r="R76" t="inlineStr"/>
       <c r="S76" t="inlineStr">
         <is>
           <t>소나무림</t>
@@ -11448,7 +11374,6 @@
       <c r="Q77" t="n">
         <v>27</v>
       </c>
-      <c r="R77" t="inlineStr"/>
       <c r="S77" t="inlineStr">
         <is>
           <t>소나무림</t>
@@ -11572,7 +11497,6 @@
       <c r="Q78" t="n">
         <v>28</v>
       </c>
-      <c r="R78" t="inlineStr"/>
       <c r="S78" t="inlineStr">
         <is>
           <t>소나무림</t>
@@ -11696,7 +11620,6 @@
       <c r="Q79" t="n">
         <v>102</v>
       </c>
-      <c r="R79" t="inlineStr"/>
       <c r="S79" t="inlineStr">
         <is>
           <t>소나무림</t>
@@ -11820,7 +11743,6 @@
       <c r="Q80" t="n">
         <v>30</v>
       </c>
-      <c r="R80" t="inlineStr"/>
       <c r="S80" t="inlineStr">
         <is>
           <t>일본잎갈나무림 a</t>
@@ -11944,7 +11866,6 @@
       <c r="Q81" t="n">
         <v>23</v>
       </c>
-      <c r="R81" t="inlineStr"/>
       <c r="S81" t="inlineStr">
         <is>
           <t>일본잎갈나무림 a</t>
@@ -12068,7 +11989,6 @@
       <c r="Q82" t="n">
         <v>51</v>
       </c>
-      <c r="R82" t="inlineStr"/>
       <c r="S82" t="inlineStr">
         <is>
           <t>일본잎갈나무림 a</t>
@@ -12192,7 +12112,6 @@
       <c r="Q83" t="n">
         <v>30</v>
       </c>
-      <c r="R83" t="inlineStr"/>
       <c r="S83" t="inlineStr">
         <is>
           <t>일본잎갈나무림 a</t>
@@ -12316,7 +12235,6 @@
       <c r="Q84" t="n">
         <v>30</v>
       </c>
-      <c r="R84" t="inlineStr"/>
       <c r="S84" t="inlineStr">
         <is>
           <t>일본잎갈나무림 a</t>
@@ -12440,7 +12358,6 @@
       <c r="Q85" t="n">
         <v>303</v>
       </c>
-      <c r="R85" t="inlineStr"/>
       <c r="S85" t="inlineStr">
         <is>
           <t>버들나무림 b</t>
@@ -12564,7 +12481,6 @@
       <c r="Q86" t="n">
         <v>57</v>
       </c>
-      <c r="R86" t="inlineStr"/>
       <c r="S86" t="inlineStr">
         <is>
           <t>버들나무림 b</t>
@@ -12688,7 +12604,6 @@
       <c r="Q87" t="n">
         <v>51</v>
       </c>
-      <c r="R87" t="inlineStr"/>
       <c r="S87" t="inlineStr">
         <is>
           <t>버들나무림 b</t>
@@ -12812,7 +12727,6 @@
       <c r="Q88" t="n">
         <v>55</v>
       </c>
-      <c r="R88" t="inlineStr"/>
       <c r="S88" t="inlineStr">
         <is>
           <t>버들나무림 b</t>
@@ -12936,7 +12850,6 @@
       <c r="Q89" t="n">
         <v>363</v>
       </c>
-      <c r="R89" t="inlineStr"/>
       <c r="S89" t="inlineStr">
         <is>
           <t>버들나무림 b</t>
@@ -13060,7 +12973,6 @@
       <c r="Q90" t="n">
         <v>150</v>
       </c>
-      <c r="R90" t="inlineStr"/>
       <c r="S90" t="inlineStr">
         <is>
           <t>일본잎갈나무림 b</t>
@@ -13184,7 +13096,6 @@
       <c r="Q91" t="n">
         <v>36</v>
       </c>
-      <c r="R91" t="inlineStr"/>
       <c r="S91" t="inlineStr">
         <is>
           <t>일본잎갈나무림 b</t>
@@ -13308,7 +13219,6 @@
       <c r="Q92" t="n">
         <v>104</v>
       </c>
-      <c r="R92" t="inlineStr"/>
       <c r="S92" t="inlineStr">
         <is>
           <t>일본잎갈나무림 b</t>
@@ -13432,7 +13342,6 @@
       <c r="Q93" t="n">
         <v>124</v>
       </c>
-      <c r="R93" t="inlineStr"/>
       <c r="S93" t="inlineStr">
         <is>
           <t>일본잎갈나무림 b</t>
@@ -13556,7 +13465,6 @@
       <c r="Q94" t="n">
         <v>159</v>
       </c>
-      <c r="R94" t="inlineStr"/>
       <c r="S94" t="inlineStr">
         <is>
           <t>일본잎갈나무림 b</t>
@@ -13680,7 +13588,6 @@
       <c r="Q95" t="n">
         <v>38</v>
       </c>
-      <c r="R95" t="inlineStr"/>
       <c r="S95" t="inlineStr">
         <is>
           <t>잣나무림 b</t>
@@ -13804,7 +13711,6 @@
       <c r="Q96" t="n">
         <v>52</v>
       </c>
-      <c r="R96" t="inlineStr"/>
       <c r="S96" t="inlineStr">
         <is>
           <t>잣나무림 b</t>
@@ -13928,7 +13834,6 @@
       <c r="Q97" t="n">
         <v>79</v>
       </c>
-      <c r="R97" t="inlineStr"/>
       <c r="S97" t="inlineStr">
         <is>
           <t>잣나무림 b</t>
@@ -14052,7 +13957,6 @@
       <c r="Q98" t="n">
         <v>34</v>
       </c>
-      <c r="R98" t="inlineStr"/>
       <c r="S98" t="inlineStr">
         <is>
           <t>잣나무림 b</t>
@@ -14176,7 +14080,6 @@
       <c r="Q99" t="n">
         <v>25</v>
       </c>
-      <c r="R99" t="inlineStr"/>
       <c r="S99" t="inlineStr">
         <is>
           <t>잣나무림 b</t>
@@ -14300,7 +14203,6 @@
       <c r="Q100" t="n">
         <v>41</v>
       </c>
-      <c r="R100" t="inlineStr"/>
       <c r="S100" t="inlineStr">
         <is>
           <t>리기다소나무림</t>
@@ -14424,7 +14326,6 @@
       <c r="Q101" t="n">
         <v>37</v>
       </c>
-      <c r="R101" t="inlineStr"/>
       <c r="S101" t="inlineStr">
         <is>
           <t>리기다소나무림</t>
@@ -14548,7 +14449,6 @@
       <c r="Q102" t="n">
         <v>42</v>
       </c>
-      <c r="R102" t="inlineStr"/>
       <c r="S102" t="inlineStr">
         <is>
           <t>리기다소나무림</t>
@@ -14672,7 +14572,6 @@
       <c r="Q103" t="n">
         <v>176</v>
       </c>
-      <c r="R103" t="inlineStr"/>
       <c r="S103" t="inlineStr">
         <is>
           <t>리기다소나무림</t>
@@ -14796,7 +14695,6 @@
       <c r="Q104" t="n">
         <v>48</v>
       </c>
-      <c r="R104" t="inlineStr"/>
       <c r="S104" t="inlineStr">
         <is>
           <t>리기다소나무림</t>
@@ -14920,7 +14818,6 @@
       <c r="Q105" t="n">
         <v>37</v>
       </c>
-      <c r="R105" t="inlineStr"/>
       <c r="S105" t="inlineStr">
         <is>
           <t>잣나무림 a</t>
@@ -15044,7 +14941,6 @@
       <c r="Q106" t="n">
         <v>144</v>
       </c>
-      <c r="R106" t="inlineStr"/>
       <c r="S106" t="inlineStr">
         <is>
           <t>잣나무림 a</t>
@@ -15168,7 +15064,6 @@
       <c r="Q107" t="n">
         <v>43</v>
       </c>
-      <c r="R107" t="inlineStr"/>
       <c r="S107" t="inlineStr">
         <is>
           <t>잣나무림 a</t>
@@ -15292,7 +15187,6 @@
       <c r="Q108" t="n">
         <v>95</v>
       </c>
-      <c r="R108" t="inlineStr"/>
       <c r="S108" t="inlineStr">
         <is>
           <t>잣나무림 a</t>
@@ -15416,7 +15310,6 @@
       <c r="Q109" t="n">
         <v>46</v>
       </c>
-      <c r="R109" t="inlineStr"/>
       <c r="S109" t="inlineStr">
         <is>
           <t>잣나무림 a</t>
@@ -15540,7 +15433,6 @@
       <c r="Q110" t="n">
         <v>56</v>
       </c>
-      <c r="R110" t="inlineStr"/>
       <c r="S110" t="inlineStr">
         <is>
           <t>버들나무림 a</t>
@@ -15664,7 +15556,6 @@
       <c r="Q111" t="n">
         <v>140</v>
       </c>
-      <c r="R111" t="inlineStr"/>
       <c r="S111" t="inlineStr">
         <is>
           <t>버들나무림 a</t>
@@ -15788,7 +15679,6 @@
       <c r="Q112" t="n">
         <v>54</v>
       </c>
-      <c r="R112" t="inlineStr"/>
       <c r="S112" t="inlineStr">
         <is>
           <t>버들나무림 a</t>
@@ -15912,7 +15802,6 @@
       <c r="Q113" t="n">
         <v>70</v>
       </c>
-      <c r="R113" t="inlineStr"/>
       <c r="S113" t="inlineStr">
         <is>
           <t>버들나무림 a</t>
@@ -16036,7 +15925,6 @@
       <c r="Q114" t="n">
         <v>47</v>
       </c>
-      <c r="R114" t="inlineStr"/>
       <c r="S114" t="inlineStr">
         <is>
           <t>버들나무림 a</t>
@@ -16160,7 +16048,6 @@
       <c r="Q115" t="n">
         <v>112</v>
       </c>
-      <c r="R115" t="inlineStr"/>
       <c r="S115" t="inlineStr">
         <is>
           <t>밭(대조구)</t>
@@ -16284,7 +16171,6 @@
       <c r="Q116" t="n">
         <v>183</v>
       </c>
-      <c r="R116" t="inlineStr"/>
       <c r="S116" t="inlineStr">
         <is>
           <t>밭(대조구)</t>
@@ -16408,7 +16294,6 @@
       <c r="Q117" t="n">
         <v>146</v>
       </c>
-      <c r="R117" t="inlineStr"/>
       <c r="S117" t="inlineStr">
         <is>
           <t>밭(대조구)</t>
@@ -16532,7 +16417,6 @@
       <c r="Q118" t="n">
         <v>95</v>
       </c>
-      <c r="R118" t="inlineStr"/>
       <c r="S118" t="inlineStr">
         <is>
           <t>밭(대조구)</t>
@@ -16656,7 +16540,6 @@
       <c r="Q119" t="n">
         <v>83</v>
       </c>
-      <c r="R119" t="inlineStr"/>
       <c r="S119" t="inlineStr">
         <is>
           <t>밭(대조구)</t>
@@ -16780,7 +16663,6 @@
       <c r="Q120" t="n">
         <v>49</v>
       </c>
-      <c r="R120" t="inlineStr"/>
       <c r="S120" t="inlineStr">
         <is>
           <t>주차장(대조구)</t>
@@ -16904,7 +16786,6 @@
       <c r="Q121" t="n">
         <v>44</v>
       </c>
-      <c r="R121" t="inlineStr"/>
       <c r="S121" t="inlineStr">
         <is>
           <t>주차장(대조구)</t>
@@ -17028,7 +16909,6 @@
       <c r="Q122" t="n">
         <v>66</v>
       </c>
-      <c r="R122" t="inlineStr"/>
       <c r="S122" t="inlineStr">
         <is>
           <t>주차장(대조구)</t>
@@ -17152,7 +17032,6 @@
       <c r="Q123" t="n">
         <v>32</v>
       </c>
-      <c r="R123" t="inlineStr"/>
       <c r="S123" t="inlineStr">
         <is>
           <t>주차장(대조구)</t>
@@ -17276,7 +17155,6 @@
       <c r="Q124" t="n">
         <v>37</v>
       </c>
-      <c r="R124" t="inlineStr"/>
       <c r="S124" t="inlineStr">
         <is>
           <t>주차장(대조구)</t>
@@ -17400,7 +17278,6 @@
       <c r="Q125" t="n">
         <v>38</v>
       </c>
-      <c r="R125" t="inlineStr"/>
       <c r="S125" t="inlineStr">
         <is>
           <t>소나무림</t>
@@ -17524,7 +17401,6 @@
       <c r="Q126" t="n">
         <v>33</v>
       </c>
-      <c r="R126" t="inlineStr"/>
       <c r="S126" t="inlineStr">
         <is>
           <t>소나무림</t>
@@ -17648,7 +17524,6 @@
       <c r="Q127" t="n">
         <v>27</v>
       </c>
-      <c r="R127" t="inlineStr"/>
       <c r="S127" t="inlineStr">
         <is>
           <t>소나무림</t>
@@ -17772,7 +17647,6 @@
       <c r="Q128" t="n">
         <v>28</v>
       </c>
-      <c r="R128" t="inlineStr"/>
       <c r="S128" t="inlineStr">
         <is>
           <t>소나무림</t>
@@ -17896,7 +17770,6 @@
       <c r="Q129" t="n">
         <v>102</v>
       </c>
-      <c r="R129" t="inlineStr"/>
       <c r="S129" t="inlineStr">
         <is>
           <t>소나무림</t>
@@ -18020,7 +17893,6 @@
       <c r="Q130" t="n">
         <v>30</v>
       </c>
-      <c r="R130" t="inlineStr"/>
       <c r="S130" t="inlineStr">
         <is>
           <t>일본잎갈나무림 a</t>
@@ -18144,7 +18016,6 @@
       <c r="Q131" t="n">
         <v>23</v>
       </c>
-      <c r="R131" t="inlineStr"/>
       <c r="S131" t="inlineStr">
         <is>
           <t>일본잎갈나무림 a</t>
@@ -18268,7 +18139,6 @@
       <c r="Q132" t="n">
         <v>51</v>
       </c>
-      <c r="R132" t="inlineStr"/>
       <c r="S132" t="inlineStr">
         <is>
           <t>일본잎갈나무림 a</t>
@@ -18392,7 +18262,6 @@
       <c r="Q133" t="n">
         <v>30</v>
       </c>
-      <c r="R133" t="inlineStr"/>
       <c r="S133" t="inlineStr">
         <is>
           <t>일본잎갈나무림 a</t>
@@ -18516,7 +18385,6 @@
       <c r="Q134" t="n">
         <v>30</v>
       </c>
-      <c r="R134" t="inlineStr"/>
       <c r="S134" t="inlineStr">
         <is>
           <t>일본잎갈나무림 a</t>
@@ -18640,7 +18508,6 @@
       <c r="Q135" t="n">
         <v>303</v>
       </c>
-      <c r="R135" t="inlineStr"/>
       <c r="S135" t="inlineStr">
         <is>
           <t>버들나무림 b</t>
@@ -18764,7 +18631,6 @@
       <c r="Q136" t="n">
         <v>57</v>
       </c>
-      <c r="R136" t="inlineStr"/>
       <c r="S136" t="inlineStr">
         <is>
           <t>버들나무림 b</t>
@@ -18888,7 +18754,6 @@
       <c r="Q137" t="n">
         <v>51</v>
       </c>
-      <c r="R137" t="inlineStr"/>
       <c r="S137" t="inlineStr">
         <is>
           <t>버들나무림 b</t>
@@ -19012,7 +18877,6 @@
       <c r="Q138" t="n">
         <v>55</v>
       </c>
-      <c r="R138" t="inlineStr"/>
       <c r="S138" t="inlineStr">
         <is>
           <t>버들나무림 b</t>
@@ -19136,7 +19000,6 @@
       <c r="Q139" t="n">
         <v>363</v>
       </c>
-      <c r="R139" t="inlineStr"/>
       <c r="S139" t="inlineStr">
         <is>
           <t>버들나무림 b</t>
@@ -19260,7 +19123,6 @@
       <c r="Q140" t="n">
         <v>150</v>
       </c>
-      <c r="R140" t="inlineStr"/>
       <c r="S140" t="inlineStr">
         <is>
           <t>일본잎갈나무림 b</t>
@@ -19384,7 +19246,6 @@
       <c r="Q141" t="n">
         <v>36</v>
       </c>
-      <c r="R141" t="inlineStr"/>
       <c r="S141" t="inlineStr">
         <is>
           <t>일본잎갈나무림 b</t>
@@ -19508,7 +19369,6 @@
       <c r="Q142" t="n">
         <v>104</v>
       </c>
-      <c r="R142" t="inlineStr"/>
       <c r="S142" t="inlineStr">
         <is>
           <t>일본잎갈나무림 b</t>
@@ -19632,7 +19492,6 @@
       <c r="Q143" t="n">
         <v>124</v>
       </c>
-      <c r="R143" t="inlineStr"/>
       <c r="S143" t="inlineStr">
         <is>
           <t>일본잎갈나무림 b</t>
@@ -19756,7 +19615,6 @@
       <c r="Q144" t="n">
         <v>159</v>
       </c>
-      <c r="R144" t="inlineStr"/>
       <c r="S144" t="inlineStr">
         <is>
           <t>일본잎갈나무림 b</t>
@@ -19880,7 +19738,6 @@
       <c r="Q145" t="n">
         <v>38</v>
       </c>
-      <c r="R145" t="inlineStr"/>
       <c r="S145" t="inlineStr">
         <is>
           <t>잣나무림 b</t>
@@ -20004,7 +19861,6 @@
       <c r="Q146" t="n">
         <v>52</v>
       </c>
-      <c r="R146" t="inlineStr"/>
       <c r="S146" t="inlineStr">
         <is>
           <t>잣나무림 b</t>
@@ -20128,7 +19984,6 @@
       <c r="Q147" t="n">
         <v>79</v>
       </c>
-      <c r="R147" t="inlineStr"/>
       <c r="S147" t="inlineStr">
         <is>
           <t>잣나무림 b</t>
@@ -20252,7 +20107,6 @@
       <c r="Q148" t="n">
         <v>34</v>
       </c>
-      <c r="R148" t="inlineStr"/>
       <c r="S148" t="inlineStr">
         <is>
           <t>잣나무림 b</t>
@@ -20376,7 +20230,6 @@
       <c r="Q149" t="n">
         <v>25</v>
       </c>
-      <c r="R149" t="inlineStr"/>
       <c r="S149" t="inlineStr">
         <is>
           <t>잣나무림 b</t>
@@ -20500,7 +20353,6 @@
       <c r="Q150" t="n">
         <v>79</v>
       </c>
-      <c r="R150" t="inlineStr"/>
       <c r="S150" t="inlineStr">
         <is>
           <t>리기다소나무림</t>
@@ -20624,7 +20476,6 @@
       <c r="Q151" t="n">
         <v>37</v>
       </c>
-      <c r="R151" t="inlineStr"/>
       <c r="S151" t="inlineStr">
         <is>
           <t>리기다소나무림</t>
@@ -20748,7 +20599,6 @@
       <c r="Q152" t="n">
         <v>74</v>
       </c>
-      <c r="R152" t="inlineStr"/>
       <c r="S152" t="inlineStr">
         <is>
           <t>리기다소나무림</t>
@@ -20872,7 +20722,6 @@
       <c r="Q153" t="n">
         <v>39</v>
       </c>
-      <c r="R153" t="inlineStr"/>
       <c r="S153" t="inlineStr">
         <is>
           <t>리기다소나무림</t>
@@ -20996,7 +20845,6 @@
       <c r="Q154" t="n">
         <v>117</v>
       </c>
-      <c r="R154" t="inlineStr"/>
       <c r="S154" t="inlineStr">
         <is>
           <t>리기다소나무림</t>
@@ -21120,7 +20968,6 @@
       <c r="Q155" t="n">
         <v>48</v>
       </c>
-      <c r="R155" t="inlineStr"/>
       <c r="S155" t="inlineStr">
         <is>
           <t>잣나무림 a</t>
@@ -21244,7 +21091,6 @@
       <c r="Q156" t="n">
         <v>59</v>
       </c>
-      <c r="R156" t="inlineStr"/>
       <c r="S156" t="inlineStr">
         <is>
           <t>잣나무림 a</t>
@@ -21368,7 +21214,6 @@
       <c r="Q157" t="n">
         <v>62</v>
       </c>
-      <c r="R157" t="inlineStr"/>
       <c r="S157" t="inlineStr">
         <is>
           <t>잣나무림 a</t>
@@ -21492,7 +21337,6 @@
       <c r="Q158" t="n">
         <v>66</v>
       </c>
-      <c r="R158" t="inlineStr"/>
       <c r="S158" t="inlineStr">
         <is>
           <t>잣나무림 a</t>
@@ -21616,7 +21460,6 @@
       <c r="Q159" t="n">
         <v>28</v>
       </c>
-      <c r="R159" t="inlineStr"/>
       <c r="S159" t="inlineStr">
         <is>
           <t>잣나무림 a</t>
@@ -21740,7 +21583,6 @@
       <c r="Q160" t="n">
         <v>160</v>
       </c>
-      <c r="R160" t="inlineStr"/>
       <c r="S160" t="inlineStr">
         <is>
           <t>버들나무림 a</t>
@@ -21864,7 +21706,6 @@
       <c r="Q161" t="n">
         <v>48</v>
       </c>
-      <c r="R161" t="inlineStr"/>
       <c r="S161" t="inlineStr">
         <is>
           <t>버들나무림 a</t>
@@ -21988,7 +21829,6 @@
       <c r="Q162" t="n">
         <v>83</v>
       </c>
-      <c r="R162" t="inlineStr"/>
       <c r="S162" t="inlineStr">
         <is>
           <t>버들나무림 a</t>
@@ -22112,7 +21952,6 @@
       <c r="Q163" t="n">
         <v>178</v>
       </c>
-      <c r="R163" t="inlineStr"/>
       <c r="S163" t="inlineStr">
         <is>
           <t>버들나무림 a</t>
@@ -22236,7 +22075,6 @@
       <c r="Q164" t="n">
         <v>146</v>
       </c>
-      <c r="R164" t="inlineStr"/>
       <c r="S164" t="inlineStr">
         <is>
           <t>버들나무림 a</t>
@@ -22360,7 +22198,6 @@
       <c r="Q165" t="n">
         <v>53</v>
       </c>
-      <c r="R165" t="inlineStr"/>
       <c r="S165" t="inlineStr">
         <is>
           <t>밭(대조구)</t>
@@ -22484,7 +22321,6 @@
       <c r="Q166" t="n">
         <v>51</v>
       </c>
-      <c r="R166" t="inlineStr"/>
       <c r="S166" t="inlineStr">
         <is>
           <t>밭(대조구)</t>
@@ -22608,7 +22444,6 @@
       <c r="Q167" t="n">
         <v>58</v>
       </c>
-      <c r="R167" t="inlineStr"/>
       <c r="S167" t="inlineStr">
         <is>
           <t>밭(대조구)</t>
@@ -22732,7 +22567,6 @@
       <c r="Q168" t="n">
         <v>58</v>
       </c>
-      <c r="R168" t="inlineStr"/>
       <c r="S168" t="inlineStr">
         <is>
           <t>밭(대조구)</t>
@@ -22856,7 +22690,6 @@
       <c r="Q169" t="n">
         <v>174</v>
       </c>
-      <c r="R169" t="inlineStr"/>
       <c r="S169" t="inlineStr">
         <is>
           <t>밭(대조구)</t>
@@ -22980,7 +22813,6 @@
       <c r="Q170" t="n">
         <v>53</v>
       </c>
-      <c r="R170" t="inlineStr"/>
       <c r="S170" t="inlineStr">
         <is>
           <t>주차장(대조구)</t>
@@ -23104,7 +22936,6 @@
       <c r="Q171" t="n">
         <v>43</v>
       </c>
-      <c r="R171" t="inlineStr"/>
       <c r="S171" t="inlineStr">
         <is>
           <t>주차장(대조구)</t>
@@ -23228,7 +23059,6 @@
       <c r="Q172" t="n">
         <v>46</v>
       </c>
-      <c r="R172" t="inlineStr"/>
       <c r="S172" t="inlineStr">
         <is>
           <t>주차장(대조구)</t>
@@ -23352,7 +23182,6 @@
       <c r="Q173" t="n">
         <v>28</v>
       </c>
-      <c r="R173" t="inlineStr"/>
       <c r="S173" t="inlineStr">
         <is>
           <t>주차장(대조구)</t>
@@ -23476,7 +23305,6 @@
       <c r="Q174" t="n">
         <v>51</v>
       </c>
-      <c r="R174" t="inlineStr"/>
       <c r="S174" t="inlineStr">
         <is>
           <t>주차장(대조구)</t>
@@ -23600,7 +23428,6 @@
       <c r="Q175" t="n">
         <v>44</v>
       </c>
-      <c r="R175" t="inlineStr"/>
       <c r="S175" t="inlineStr">
         <is>
           <t>소나무림</t>
@@ -23724,7 +23551,6 @@
       <c r="Q176" t="n">
         <v>112</v>
       </c>
-      <c r="R176" t="inlineStr"/>
       <c r="S176" t="inlineStr">
         <is>
           <t>소나무림</t>
@@ -23848,7 +23674,6 @@
       <c r="Q177" t="n">
         <v>55</v>
       </c>
-      <c r="R177" t="inlineStr"/>
       <c r="S177" t="inlineStr">
         <is>
           <t>소나무림</t>
@@ -23972,7 +23797,6 @@
       <c r="Q178" t="n">
         <v>36</v>
       </c>
-      <c r="R178" t="inlineStr"/>
       <c r="S178" t="inlineStr">
         <is>
           <t>소나무림</t>
@@ -24096,7 +23920,6 @@
       <c r="Q179" t="n">
         <v>75</v>
       </c>
-      <c r="R179" t="inlineStr"/>
       <c r="S179" t="inlineStr">
         <is>
           <t>소나무림</t>
@@ -24220,7 +24043,6 @@
       <c r="Q180" t="n">
         <v>45</v>
       </c>
-      <c r="R180" t="inlineStr"/>
       <c r="S180" t="inlineStr">
         <is>
           <t>일본잎갈나무림 a</t>
@@ -24344,7 +24166,6 @@
       <c r="Q181" t="n">
         <v>45</v>
       </c>
-      <c r="R181" t="inlineStr"/>
       <c r="S181" t="inlineStr">
         <is>
           <t>일본잎갈나무림 a</t>
@@ -24468,7 +24289,6 @@
       <c r="Q182" t="n">
         <v>64</v>
       </c>
-      <c r="R182" t="inlineStr"/>
       <c r="S182" t="inlineStr">
         <is>
           <t>일본잎갈나무림 a</t>
@@ -24592,7 +24412,6 @@
       <c r="Q183" t="n">
         <v>45</v>
       </c>
-      <c r="R183" t="inlineStr"/>
       <c r="S183" t="inlineStr">
         <is>
           <t>일본잎갈나무림 a</t>
@@ -24716,7 +24535,6 @@
       <c r="Q184" t="n">
         <v>81</v>
       </c>
-      <c r="R184" t="inlineStr"/>
       <c r="S184" t="inlineStr">
         <is>
           <t>일본잎갈나무림 a</t>
@@ -24840,7 +24658,6 @@
       <c r="Q185" t="n">
         <v>143</v>
       </c>
-      <c r="R185" t="inlineStr"/>
       <c r="S185" t="inlineStr">
         <is>
           <t>버들나무림 b</t>
@@ -24964,7 +24781,6 @@
       <c r="Q186" t="n">
         <v>60</v>
       </c>
-      <c r="R186" t="inlineStr"/>
       <c r="S186" t="inlineStr">
         <is>
           <t>버들나무림 b</t>
@@ -25088,7 +24904,6 @@
       <c r="Q187" t="n">
         <v>206</v>
       </c>
-      <c r="R187" t="inlineStr"/>
       <c r="S187" t="inlineStr">
         <is>
           <t>버들나무림 b</t>
@@ -25212,7 +25027,6 @@
       <c r="Q188" t="n">
         <v>115</v>
       </c>
-      <c r="R188" t="inlineStr"/>
       <c r="S188" t="inlineStr">
         <is>
           <t>버들나무림 b</t>
@@ -25336,7 +25150,6 @@
       <c r="Q189" t="n">
         <v>74</v>
       </c>
-      <c r="R189" t="inlineStr"/>
       <c r="S189" t="inlineStr">
         <is>
           <t>버들나무림 b</t>
@@ -25460,7 +25273,6 @@
       <c r="Q190" t="n">
         <v>228</v>
       </c>
-      <c r="R190" t="inlineStr"/>
       <c r="S190" t="inlineStr">
         <is>
           <t>일본잎갈나무림 b</t>
@@ -25584,7 +25396,6 @@
       <c r="Q191" t="n">
         <v>174</v>
       </c>
-      <c r="R191" t="inlineStr"/>
       <c r="S191" t="inlineStr">
         <is>
           <t>일본잎갈나무림 b</t>
@@ -25708,7 +25519,6 @@
       <c r="Q192" t="n">
         <v>100</v>
       </c>
-      <c r="R192" t="inlineStr"/>
       <c r="S192" t="inlineStr">
         <is>
           <t>일본잎갈나무림 b</t>
@@ -25832,7 +25642,6 @@
       <c r="Q193" t="n">
         <v>106</v>
       </c>
-      <c r="R193" t="inlineStr"/>
       <c r="S193" t="inlineStr">
         <is>
           <t>일본잎갈나무림 b</t>
@@ -25956,7 +25765,6 @@
       <c r="Q194" t="n">
         <v>283</v>
       </c>
-      <c r="R194" t="inlineStr"/>
       <c r="S194" t="inlineStr">
         <is>
           <t>일본잎갈나무림 b</t>
@@ -26080,7 +25888,6 @@
       <c r="Q195" t="n">
         <v>23</v>
       </c>
-      <c r="R195" t="inlineStr"/>
       <c r="S195" t="inlineStr">
         <is>
           <t>잣나무림 b</t>
@@ -26204,7 +26011,6 @@
       <c r="Q196" t="n">
         <v>78</v>
       </c>
-      <c r="R196" t="inlineStr"/>
       <c r="S196" t="inlineStr">
         <is>
           <t>잣나무림 b</t>
@@ -26328,7 +26134,6 @@
       <c r="Q197" t="n">
         <v>29</v>
       </c>
-      <c r="R197" t="inlineStr"/>
       <c r="S197" t="inlineStr">
         <is>
           <t>잣나무림 b</t>
@@ -26452,7 +26257,6 @@
       <c r="Q198" t="n">
         <v>42</v>
       </c>
-      <c r="R198" t="inlineStr"/>
       <c r="S198" t="inlineStr">
         <is>
           <t>잣나무림 b</t>
@@ -26576,7 +26380,6 @@
       <c r="Q199" t="n">
         <v>61</v>
       </c>
-      <c r="R199" t="inlineStr"/>
       <c r="S199" t="inlineStr">
         <is>
           <t>잣나무림 b</t>
@@ -26700,7 +26503,6 @@
       <c r="Q200" t="n">
         <v>17</v>
       </c>
-      <c r="R200" t="inlineStr"/>
       <c r="S200" t="inlineStr">
         <is>
           <t>리기다소나무림</t>
@@ -26824,7 +26626,6 @@
       <c r="Q201" t="n">
         <v>1</v>
       </c>
-      <c r="R201" t="inlineStr"/>
       <c r="S201" t="inlineStr">
         <is>
           <t>리기다소나무림</t>
@@ -26948,7 +26749,6 @@
       <c r="Q202" t="n">
         <v>114</v>
       </c>
-      <c r="R202" t="inlineStr"/>
       <c r="S202" t="inlineStr">
         <is>
           <t>리기다소나무림</t>
@@ -27072,7 +26872,6 @@
       <c r="Q203" t="n">
         <v>69</v>
       </c>
-      <c r="R203" t="inlineStr"/>
       <c r="S203" t="inlineStr">
         <is>
           <t>리기다소나무림</t>
@@ -27196,7 +26995,6 @@
       <c r="Q204" t="n">
         <v>47</v>
       </c>
-      <c r="R204" t="inlineStr"/>
       <c r="S204" t="inlineStr">
         <is>
           <t>리기다소나무림</t>
@@ -27320,7 +27118,6 @@
       <c r="Q205" t="n">
         <v>129</v>
       </c>
-      <c r="R205" t="inlineStr"/>
       <c r="S205" t="inlineStr">
         <is>
           <t>잣나무림 a</t>
@@ -27444,7 +27241,6 @@
       <c r="Q206" t="n">
         <v>569</v>
       </c>
-      <c r="R206" t="inlineStr"/>
       <c r="S206" t="inlineStr">
         <is>
           <t>잣나무림 a</t>
@@ -27568,7 +27364,6 @@
       <c r="Q207" t="n">
         <v>77</v>
       </c>
-      <c r="R207" t="inlineStr"/>
       <c r="S207" t="inlineStr">
         <is>
           <t>잣나무림 a</t>
@@ -27692,7 +27487,6 @@
       <c r="Q208" t="n">
         <v>124</v>
       </c>
-      <c r="R208" t="inlineStr"/>
       <c r="S208" t="inlineStr">
         <is>
           <t>잣나무림 a</t>
@@ -27816,7 +27610,6 @@
       <c r="Q209" t="n">
         <v>153</v>
       </c>
-      <c r="R209" t="inlineStr"/>
       <c r="S209" t="inlineStr">
         <is>
           <t>잣나무림 a</t>
@@ -27940,7 +27733,6 @@
       <c r="Q210" t="n">
         <v>79</v>
       </c>
-      <c r="R210" t="inlineStr"/>
       <c r="S210" t="inlineStr">
         <is>
           <t>버들나무림 a</t>
@@ -28064,7 +27856,6 @@
       <c r="Q211" t="n">
         <v>159</v>
       </c>
-      <c r="R211" t="inlineStr"/>
       <c r="S211" t="inlineStr">
         <is>
           <t>버들나무림 a</t>
@@ -28188,7 +27979,6 @@
       <c r="Q212" t="n">
         <v>53</v>
       </c>
-      <c r="R212" t="inlineStr"/>
       <c r="S212" t="inlineStr">
         <is>
           <t>버들나무림 a</t>
@@ -28312,7 +28102,6 @@
       <c r="Q213" t="n">
         <v>356</v>
       </c>
-      <c r="R213" t="inlineStr"/>
       <c r="S213" t="inlineStr">
         <is>
           <t>버들나무림 a</t>
@@ -28436,7 +28225,6 @@
       <c r="Q214" t="n">
         <v>189</v>
       </c>
-      <c r="R214" t="inlineStr"/>
       <c r="S214" t="inlineStr">
         <is>
           <t>버들나무림 a</t>
@@ -28560,7 +28348,6 @@
       <c r="Q215" t="n">
         <v>368</v>
       </c>
-      <c r="R215" t="inlineStr"/>
       <c r="S215" t="inlineStr">
         <is>
           <t>밭(대조구)</t>
@@ -28684,7 +28471,6 @@
       <c r="Q216" t="n">
         <v>202</v>
       </c>
-      <c r="R216" t="inlineStr"/>
       <c r="S216" t="inlineStr">
         <is>
           <t>밭(대조구)</t>
@@ -28808,7 +28594,6 @@
       <c r="Q217" t="n">
         <v>309</v>
       </c>
-      <c r="R217" t="inlineStr"/>
       <c r="S217" t="inlineStr">
         <is>
           <t>밭(대조구)</t>
@@ -28932,7 +28717,6 @@
       <c r="Q218" t="n">
         <v>234</v>
       </c>
-      <c r="R218" t="inlineStr"/>
       <c r="S218" t="inlineStr">
         <is>
           <t>밭(대조구)</t>
@@ -29056,7 +28840,6 @@
       <c r="Q219" t="n">
         <v>119</v>
       </c>
-      <c r="R219" t="inlineStr"/>
       <c r="S219" t="inlineStr">
         <is>
           <t>밭(대조구)</t>
@@ -29180,7 +28963,6 @@
       <c r="Q220" t="n">
         <v>57</v>
       </c>
-      <c r="R220" t="inlineStr"/>
       <c r="S220" t="inlineStr">
         <is>
           <t>주차장(대조구)</t>
@@ -29304,7 +29086,6 @@
       <c r="Q221" t="n">
         <v>6</v>
       </c>
-      <c r="R221" t="inlineStr"/>
       <c r="S221" t="inlineStr">
         <is>
           <t>주차장(대조구)</t>
@@ -29428,7 +29209,6 @@
       <c r="Q222" t="n">
         <v>44</v>
       </c>
-      <c r="R222" t="inlineStr"/>
       <c r="S222" t="inlineStr">
         <is>
           <t>주차장(대조구)</t>
@@ -29552,7 +29332,6 @@
       <c r="Q223" t="n">
         <v>47</v>
       </c>
-      <c r="R223" t="inlineStr"/>
       <c r="S223" t="inlineStr">
         <is>
           <t>주차장(대조구)</t>
@@ -29676,7 +29455,6 @@
       <c r="Q224" t="n">
         <v>9</v>
       </c>
-      <c r="R224" t="inlineStr"/>
       <c r="S224" t="inlineStr">
         <is>
           <t>주차장(대조구)</t>
@@ -29800,7 +29578,6 @@
       <c r="Q225" t="n">
         <v>62</v>
       </c>
-      <c r="R225" t="inlineStr"/>
       <c r="S225" t="inlineStr">
         <is>
           <t>소나무림</t>
@@ -29924,7 +29701,6 @@
       <c r="Q226" t="n">
         <v>234</v>
       </c>
-      <c r="R226" t="inlineStr"/>
       <c r="S226" t="inlineStr">
         <is>
           <t>소나무림</t>
@@ -30048,7 +29824,6 @@
       <c r="Q227" t="n">
         <v>17</v>
       </c>
-      <c r="R227" t="inlineStr"/>
       <c r="S227" t="inlineStr">
         <is>
           <t>소나무림</t>
@@ -30172,7 +29947,6 @@
       <c r="Q228" t="n">
         <v>49</v>
       </c>
-      <c r="R228" t="inlineStr"/>
       <c r="S228" t="inlineStr">
         <is>
           <t>소나무림</t>
@@ -30296,7 +30070,6 @@
       <c r="Q229" t="n">
         <v>13</v>
       </c>
-      <c r="R229" t="inlineStr"/>
       <c r="S229" t="inlineStr">
         <is>
           <t>소나무림</t>
@@ -30420,7 +30193,6 @@
       <c r="Q230" t="n">
         <v>58</v>
       </c>
-      <c r="R230" t="inlineStr"/>
       <c r="S230" t="inlineStr">
         <is>
           <t>일본잎갈나무림 a</t>
@@ -30544,7 +30316,6 @@
       <c r="Q231" t="n">
         <v>77</v>
       </c>
-      <c r="R231" t="inlineStr"/>
       <c r="S231" t="inlineStr">
         <is>
           <t>일본잎갈나무림 a</t>
@@ -30668,7 +30439,6 @@
       <c r="Q232" t="n">
         <v>55</v>
       </c>
-      <c r="R232" t="inlineStr"/>
       <c r="S232" t="inlineStr">
         <is>
           <t>일본잎갈나무림 a</t>
@@ -30792,7 +30562,6 @@
       <c r="Q233" t="n">
         <v>85</v>
       </c>
-      <c r="R233" t="inlineStr"/>
       <c r="S233" t="inlineStr">
         <is>
           <t>일본잎갈나무림 a</t>
@@ -30916,7 +30685,6 @@
       <c r="Q234" t="n">
         <v>45</v>
       </c>
-      <c r="R234" t="inlineStr"/>
       <c r="S234" t="inlineStr">
         <is>
           <t>일본잎갈나무림 a</t>
@@ -31040,7 +30808,6 @@
       <c r="Q235" t="n">
         <v>59</v>
       </c>
-      <c r="R235" t="inlineStr"/>
       <c r="S235" t="inlineStr">
         <is>
           <t>버들나무림 b</t>
@@ -31164,7 +30931,6 @@
       <c r="Q236" t="n">
         <v>281</v>
       </c>
-      <c r="R236" t="inlineStr"/>
       <c r="S236" t="inlineStr">
         <is>
           <t>버들나무림 b</t>
@@ -31288,7 +31054,6 @@
       <c r="Q237" t="n">
         <v>113</v>
       </c>
-      <c r="R237" t="inlineStr"/>
       <c r="S237" t="inlineStr">
         <is>
           <t>버들나무림 b</t>
@@ -31412,7 +31177,6 @@
       <c r="Q238" t="n">
         <v>47</v>
       </c>
-      <c r="R238" t="inlineStr"/>
       <c r="S238" t="inlineStr">
         <is>
           <t>버들나무림 b</t>
@@ -31536,7 +31300,6 @@
       <c r="Q239" t="n">
         <v>149</v>
       </c>
-      <c r="R239" t="inlineStr"/>
       <c r="S239" t="inlineStr">
         <is>
           <t>버들나무림 b</t>
@@ -31660,7 +31423,6 @@
       <c r="Q240" t="n">
         <v>43</v>
       </c>
-      <c r="R240" t="inlineStr"/>
       <c r="S240" t="inlineStr">
         <is>
           <t>일본잎갈나무림 b</t>
@@ -31784,7 +31546,6 @@
       <c r="Q241" t="n">
         <v>33</v>
       </c>
-      <c r="R241" t="inlineStr"/>
       <c r="S241" t="inlineStr">
         <is>
           <t>일본잎갈나무림 b</t>
@@ -31908,7 +31669,6 @@
       <c r="Q242" t="n">
         <v>34</v>
       </c>
-      <c r="R242" t="inlineStr"/>
       <c r="S242" t="inlineStr">
         <is>
           <t>일본잎갈나무림 b</t>
@@ -32032,7 +31792,6 @@
       <c r="Q243" t="n">
         <v>122</v>
       </c>
-      <c r="R243" t="inlineStr"/>
       <c r="S243" t="inlineStr">
         <is>
           <t>일본잎갈나무림 b</t>
@@ -32156,7 +31915,6 @@
       <c r="Q244" t="n">
         <v>4</v>
       </c>
-      <c r="R244" t="inlineStr"/>
       <c r="S244" t="inlineStr">
         <is>
           <t>일본잎갈나무림 b</t>
@@ -32280,7 +32038,6 @@
       <c r="Q245" t="n">
         <v>56</v>
       </c>
-      <c r="R245" t="inlineStr"/>
       <c r="S245" t="inlineStr">
         <is>
           <t>잣나무림 b</t>
@@ -32404,7 +32161,6 @@
       <c r="Q246" t="n">
         <v>75</v>
       </c>
-      <c r="R246" t="inlineStr"/>
       <c r="S246" t="inlineStr">
         <is>
           <t>잣나무림 b</t>
@@ -32528,7 +32284,6 @@
       <c r="Q247" t="n">
         <v>59</v>
       </c>
-      <c r="R247" t="inlineStr"/>
       <c r="S247" t="inlineStr">
         <is>
           <t>잣나무림 b</t>
@@ -32652,7 +32407,6 @@
       <c r="Q248" t="n">
         <v>78</v>
       </c>
-      <c r="R248" t="inlineStr"/>
       <c r="S248" t="inlineStr">
         <is>
           <t>잣나무림 b</t>
@@ -32776,7 +32530,6 @@
       <c r="Q249" t="n">
         <v>51</v>
       </c>
-      <c r="R249" t="inlineStr"/>
       <c r="S249" t="inlineStr">
         <is>
           <t>잣나무림 b</t>
@@ -32900,7 +32653,6 @@
       <c r="Q250" t="n">
         <v>71</v>
       </c>
-      <c r="R250" t="inlineStr"/>
       <c r="S250" t="inlineStr">
         <is>
           <t>리기다소나무림</t>
@@ -33024,7 +32776,6 @@
       <c r="Q251" t="n">
         <v>29</v>
       </c>
-      <c r="R251" t="inlineStr"/>
       <c r="S251" t="inlineStr">
         <is>
           <t>리기다소나무림</t>
@@ -33148,7 +32899,6 @@
       <c r="Q252" t="n">
         <v>24</v>
       </c>
-      <c r="R252" t="inlineStr"/>
       <c r="S252" t="inlineStr">
         <is>
           <t>리기다소나무림</t>
@@ -33272,7 +33022,6 @@
       <c r="Q253" t="n">
         <v>66</v>
       </c>
-      <c r="R253" t="inlineStr"/>
       <c r="S253" t="inlineStr">
         <is>
           <t>리기다소나무림</t>
@@ -33396,7 +33145,6 @@
       <c r="Q254" t="n">
         <v>44</v>
       </c>
-      <c r="R254" t="inlineStr"/>
       <c r="S254" t="inlineStr">
         <is>
           <t>리기다소나무림</t>
@@ -33520,7 +33268,6 @@
       <c r="Q255" t="n">
         <v>45</v>
       </c>
-      <c r="R255" t="inlineStr"/>
       <c r="S255" t="inlineStr">
         <is>
           <t>잣나무림 a</t>
@@ -33644,7 +33391,6 @@
       <c r="Q256" t="n">
         <v>68</v>
       </c>
-      <c r="R256" t="inlineStr"/>
       <c r="S256" t="inlineStr">
         <is>
           <t>잣나무림 a</t>
@@ -33768,7 +33514,6 @@
       <c r="Q257" t="n">
         <v>89</v>
       </c>
-      <c r="R257" t="inlineStr"/>
       <c r="S257" t="inlineStr">
         <is>
           <t>잣나무림 a</t>
@@ -33892,7 +33637,6 @@
       <c r="Q258" t="n">
         <v>173</v>
       </c>
-      <c r="R258" t="inlineStr"/>
       <c r="S258" t="inlineStr">
         <is>
           <t>잣나무림 a</t>
@@ -34016,7 +33760,6 @@
       <c r="Q259" t="n">
         <v>155</v>
       </c>
-      <c r="R259" t="inlineStr"/>
       <c r="S259" t="inlineStr">
         <is>
           <t>잣나무림 a</t>
@@ -34140,7 +33883,6 @@
       <c r="Q260" t="n">
         <v>107</v>
       </c>
-      <c r="R260" t="inlineStr"/>
       <c r="S260" t="inlineStr">
         <is>
           <t>버들나무림 a</t>
@@ -34264,7 +34006,6 @@
       <c r="Q261" t="n">
         <v>199</v>
       </c>
-      <c r="R261" t="inlineStr"/>
       <c r="S261" t="inlineStr">
         <is>
           <t>버들나무림 a</t>
@@ -34388,7 +34129,6 @@
       <c r="Q262" t="n">
         <v>197</v>
       </c>
-      <c r="R262" t="inlineStr"/>
       <c r="S262" t="inlineStr">
         <is>
           <t>버들나무림 a</t>
@@ -34512,7 +34252,6 @@
       <c r="Q263" t="n">
         <v>102</v>
       </c>
-      <c r="R263" t="inlineStr"/>
       <c r="S263" t="inlineStr">
         <is>
           <t>버들나무림 a</t>
@@ -34636,7 +34375,6 @@
       <c r="Q264" t="n">
         <v>121</v>
       </c>
-      <c r="R264" t="inlineStr"/>
       <c r="S264" t="inlineStr">
         <is>
           <t>버들나무림 a</t>
@@ -34760,7 +34498,6 @@
       <c r="Q265" t="n">
         <v>34</v>
       </c>
-      <c r="R265" t="inlineStr"/>
       <c r="S265" t="inlineStr">
         <is>
           <t>밭(대조구)</t>
@@ -34884,7 +34621,6 @@
       <c r="Q266" t="n">
         <v>116</v>
       </c>
-      <c r="R266" t="inlineStr"/>
       <c r="S266" t="inlineStr">
         <is>
           <t>밭(대조구)</t>
@@ -35008,7 +34744,6 @@
       <c r="Q267" t="n">
         <v>175</v>
       </c>
-      <c r="R267" t="inlineStr"/>
       <c r="S267" t="inlineStr">
         <is>
           <t>밭(대조구)</t>
@@ -35132,7 +34867,6 @@
       <c r="Q268" t="n">
         <v>161</v>
       </c>
-      <c r="R268" t="inlineStr"/>
       <c r="S268" t="inlineStr">
         <is>
           <t>밭(대조구)</t>
@@ -35256,7 +34990,6 @@
       <c r="Q269" t="n">
         <v>260</v>
       </c>
-      <c r="R269" t="inlineStr"/>
       <c r="S269" t="inlineStr">
         <is>
           <t>밭(대조구)</t>
@@ -35380,7 +35113,6 @@
       <c r="Q270" t="n">
         <v>28</v>
       </c>
-      <c r="R270" t="inlineStr"/>
       <c r="S270" t="inlineStr">
         <is>
           <t>주차장(대조구)</t>
@@ -35504,7 +35236,6 @@
       <c r="Q271" t="n">
         <v>17</v>
       </c>
-      <c r="R271" t="inlineStr"/>
       <c r="S271" t="inlineStr">
         <is>
           <t>주차장(대조구)</t>
@@ -35628,7 +35359,6 @@
       <c r="Q272" t="n">
         <v>54</v>
       </c>
-      <c r="R272" t="inlineStr"/>
       <c r="S272" t="inlineStr">
         <is>
           <t>주차장(대조구)</t>
@@ -35752,7 +35482,6 @@
       <c r="Q273" t="n">
         <v>36</v>
       </c>
-      <c r="R273" t="inlineStr"/>
       <c r="S273" t="inlineStr">
         <is>
           <t>주차장(대조구)</t>
@@ -35876,7 +35605,6 @@
       <c r="Q274" t="n">
         <v>28</v>
       </c>
-      <c r="R274" t="inlineStr"/>
       <c r="S274" t="inlineStr">
         <is>
           <t>주차장(대조구)</t>
@@ -36000,7 +35728,6 @@
       <c r="Q275" t="n">
         <v>80</v>
       </c>
-      <c r="R275" t="inlineStr"/>
       <c r="S275" t="inlineStr">
         <is>
           <t>소나무림</t>
@@ -36124,7 +35851,6 @@
       <c r="Q276" t="n">
         <v>105</v>
       </c>
-      <c r="R276" t="inlineStr"/>
       <c r="S276" t="inlineStr">
         <is>
           <t>소나무림</t>
@@ -36248,7 +35974,6 @@
       <c r="Q277" t="n">
         <v>75</v>
       </c>
-      <c r="R277" t="inlineStr"/>
       <c r="S277" t="inlineStr">
         <is>
           <t>소나무림</t>
@@ -36372,7 +36097,6 @@
       <c r="Q278" t="n">
         <v>47</v>
       </c>
-      <c r="R278" t="inlineStr"/>
       <c r="S278" t="inlineStr">
         <is>
           <t>소나무림</t>
@@ -36496,7 +36220,6 @@
       <c r="Q279" t="n">
         <v>66</v>
       </c>
-      <c r="R279" t="inlineStr"/>
       <c r="S279" t="inlineStr">
         <is>
           <t>소나무림</t>
@@ -36620,7 +36343,6 @@
       <c r="Q280" t="n">
         <v>38</v>
       </c>
-      <c r="R280" t="inlineStr"/>
       <c r="S280" t="inlineStr">
         <is>
           <t>일본잎갈나무림 a</t>
@@ -36744,7 +36466,6 @@
       <c r="Q281" t="n">
         <v>56</v>
       </c>
-      <c r="R281" t="inlineStr"/>
       <c r="S281" t="inlineStr">
         <is>
           <t>일본잎갈나무림 a</t>
@@ -36868,7 +36589,6 @@
       <c r="Q282" t="n">
         <v>33</v>
       </c>
-      <c r="R282" t="inlineStr"/>
       <c r="S282" t="inlineStr">
         <is>
           <t>일본잎갈나무림 a</t>
@@ -36992,7 +36712,6 @@
       <c r="Q283" t="n">
         <v>90</v>
       </c>
-      <c r="R283" t="inlineStr"/>
       <c r="S283" t="inlineStr">
         <is>
           <t>일본잎갈나무림 a</t>
@@ -37116,7 +36835,6 @@
       <c r="Q284" t="n">
         <v>39</v>
       </c>
-      <c r="R284" t="inlineStr"/>
       <c r="S284" t="inlineStr">
         <is>
           <t>일본잎갈나무림 a</t>
@@ -37240,7 +36958,6 @@
       <c r="Q285" t="n">
         <v>71</v>
       </c>
-      <c r="R285" t="inlineStr"/>
       <c r="S285" t="inlineStr">
         <is>
           <t>버들나무림 b</t>
@@ -37364,7 +37081,6 @@
       <c r="Q286" t="n">
         <v>49</v>
       </c>
-      <c r="R286" t="inlineStr"/>
       <c r="S286" t="inlineStr">
         <is>
           <t>버들나무림 b</t>
@@ -37488,7 +37204,6 @@
       <c r="Q287" t="n">
         <v>88</v>
       </c>
-      <c r="R287" t="inlineStr"/>
       <c r="S287" t="inlineStr">
         <is>
           <t>버들나무림 b</t>
@@ -37612,7 +37327,6 @@
       <c r="Q288" t="n">
         <v>41</v>
       </c>
-      <c r="R288" t="inlineStr"/>
       <c r="S288" t="inlineStr">
         <is>
           <t>버들나무림 b</t>
@@ -37736,7 +37450,6 @@
       <c r="Q289" t="n">
         <v>114</v>
       </c>
-      <c r="R289" t="inlineStr"/>
       <c r="S289" t="inlineStr">
         <is>
           <t>버들나무림 b</t>
@@ -37860,7 +37573,6 @@
       <c r="Q290" t="n">
         <v>65</v>
       </c>
-      <c r="R290" t="inlineStr"/>
       <c r="S290" t="inlineStr">
         <is>
           <t>일본잎갈나무림 b</t>
@@ -37984,7 +37696,6 @@
       <c r="Q291" t="n">
         <v>64</v>
       </c>
-      <c r="R291" t="inlineStr"/>
       <c r="S291" t="inlineStr">
         <is>
           <t>일본잎갈나무림 b</t>
@@ -38108,7 +37819,6 @@
       <c r="Q292" t="n">
         <v>63</v>
       </c>
-      <c r="R292" t="inlineStr"/>
       <c r="S292" t="inlineStr">
         <is>
           <t>일본잎갈나무림 b</t>
@@ -38232,7 +37942,6 @@
       <c r="Q293" t="n">
         <v>77</v>
       </c>
-      <c r="R293" t="inlineStr"/>
       <c r="S293" t="inlineStr">
         <is>
           <t>일본잎갈나무림 b</t>
@@ -38356,7 +38065,6 @@
       <c r="Q294" t="n">
         <v>57</v>
       </c>
-      <c r="R294" t="inlineStr"/>
       <c r="S294" t="inlineStr">
         <is>
           <t>일본잎갈나무림 b</t>
@@ -38480,7 +38188,6 @@
       <c r="Q295" t="n">
         <v>61</v>
       </c>
-      <c r="R295" t="inlineStr"/>
       <c r="S295" t="inlineStr">
         <is>
           <t>잣나무림 b</t>
@@ -38604,7 +38311,6 @@
       <c r="Q296" t="n">
         <v>57</v>
       </c>
-      <c r="R296" t="inlineStr"/>
       <c r="S296" t="inlineStr">
         <is>
           <t>잣나무림 b</t>
@@ -38728,7 +38434,6 @@
       <c r="Q297" t="n">
         <v>74</v>
       </c>
-      <c r="R297" t="inlineStr"/>
       <c r="S297" t="inlineStr">
         <is>
           <t>잣나무림 b</t>
@@ -38852,7 +38557,6 @@
       <c r="Q298" t="n">
         <v>85</v>
       </c>
-      <c r="R298" t="inlineStr"/>
       <c r="S298" t="inlineStr">
         <is>
           <t>잣나무림 b</t>
@@ -38976,7 +38680,6 @@
       <c r="Q299" t="n">
         <v>179</v>
       </c>
-      <c r="R299" t="inlineStr"/>
       <c r="S299" t="inlineStr">
         <is>
           <t>잣나무림 b</t>
@@ -41087,6 +40790,802 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Site_No</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Stand_Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Scientific_Name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Stand_Category</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Topography</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Soil_pH</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Soil_Moisture_Pct</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>TAF_Mean_CFU</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>TAB_Mean_CFU</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>TAF_Peak_Season</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>TAF_Summer_CFU</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>DNA_Spring_Dominant</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>DNA_Summer_Dominant</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Microbial_Characteristics</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Ecological_Interpretation</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Forest_Therapy_Health</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>리기다소나무림</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Pinus rigida Mill.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>인공 침엽수 조림지</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>학술림 하단 완경사 산록부</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="G2" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="H2" t="n">
+        <v>561</v>
+      </c>
+      <c r="I2" t="n">
+        <v>14</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>4월 봄철 (688 CFU/㎥)</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>496</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Capnodiales_sp (36.6%), Penicillium_sp (25.1%), Nectriaceae_sp (10.4%), Cladosporium (10.1%)</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Trichoderma_sp (99.9% 독점 우점)</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>송진(테르펜) 함유 솔잎 낙엽층의 완만한 분해 특성. 여름철 고온다습기에 Trichoderma가 99.9%로 단일 극우점하여 토양 유기물 분해를 독점.</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>척박지 녹화용으로 조림된 리기다소나무는 산성 토양과 두터운 침엽수 낙엽 매트층을 형성함. 셀룰로오스 분해 사상균의 서식처이며 토양 병원균 증식을 억제하는 생물방제 길항 미생물상 구축.</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>솔잎 테르펜 피톤치드 효과가 우수함. 4월 건조 강풍기에는 엽면 부유 포자가 다소 증가하므로 알레르기 민감군은 보건용 마스크 착용 권장.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>잣나무림 a</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Pinus koraiensis Siebold &amp; Zucc. (Stand A)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>울창한 천연/인공 침엽수림</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>계곡 인접 완경사지, 수관 울폐도 85% 이상</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="G3" t="n">
+        <v>37.8</v>
+      </c>
+      <c r="H3" t="n">
+        <v>893.7</v>
+      </c>
+      <c r="I3" t="n">
+        <v>36.3</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>7월 한여름 (2,104 CFU/㎥, 전 지점 2위)</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>2104</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Cladosporium (41.3%), Capnodiales (27.9%), Alternaria (21.9%)</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Trichoderma (75.0%), Bjerkandera (13.7%), Penicillium (7.1%), Coprinellus (1.0%)</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>봄철 4대 알레르겐(Cladosporium, Alternaria 등 63.2%) 우점에서 여름철 고온다습기 Trichoderma(75%) 및 목재부후균 Bjerkandera(13.7%)로의 극적 천이.</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>고밀도 잣나무 수관이 하층 습도를 보존하여 낙엽층 부식이 왕성함. 여름철 다우기 직후(강우 64.6mm) 토양 셀룰로오스 분해균과 버섯 균사가 대량 번식하여 생태계 양분 순환을 가속.</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>여름철 다습기에는 포자 밀도가 2,000 CFU/㎥를 초과하므로, 중증 천식 환자는 다우 직후 체류를 자제하고 통풍이 원활한 능선부(Site 10) 이용 권장.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>버들나무림 a (왕버들 a)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Salix koreensis Andersson (Stand A)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>수변 저습지 활엽수림</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>계곡 수변부 및 저습지, 상시 물안개</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="G4" t="n">
+        <v>42.1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1087.8</v>
+      </c>
+      <c r="I4" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>7월 한여름 (1,672 CFU/㎥), 8월 (1,452 CFU/㎥)</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>1672</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Capnodiales (50.1%), Cladosporium (29.2%), Septotinia (3.2%), Fusarium (3.1%)</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Trichoderma (78.0%), Fusarium (10.2%), Coprinellus (3.1%), Clonostachys (2.9%)</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>연중 700~1,670 CFU/㎥의 지속적 고농도 유지. 수변 고습 환경과 활엽수 엽면 조직 특이적 수목 병원성 및 부생 사상균 우점.</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>하천 변 수분 포화 토양과 활엽수 연약 잎 조직으로 인해 분해 및 병원성 진균의 활성이 연중 지속됨. 수변 완충 식생의 수질 정화 및 미기후 습도 유지 생태 기능 수행.</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>수변 음이온과 습도가 풍부하나 곰팡이 과민성 비염 환자는 여름철 장시간 체류 시 비염 악화 가능성 유의.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>밭 (개활 경작지 대조구)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Agricultural Cultivated Field (Control)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>인위적 개활 경작지 (대조구)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>학술림 진입부 경작지, 수관 0% 완전 개활</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="G5" t="n">
+        <v>31</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1217.7</v>
+      </c>
+      <c r="I5" t="n">
+        <v>144.3</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>7월 한여름 (2,464 CFU/㎥, 전 지점 연중 최고)</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>2464</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>미포집 (하절기 집중 관측)</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Fusarium oxysporum (45.1%), Penicillium (32.5%), Aspergillus (10.4%), Nectriaceae (7.6%)</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>토양 서식 식물 시들음병균인 Fusarium oxysporum(45.1%)과 저장 사상균 Penicillium/Aspergillus(42.9%)가 지표면 비산 먼지와 함께 대량 방출.</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>자연 수관 부재 및 잦은 영농 토양 경운으로 지표면이 불안정하며, 시비 유기물에 의해 기회주의적 부생 곰팡이가 폭발적으로 증식하는 '인위적 교란 지표'.</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Fusarium의 곰팡이독소(Fumonisin, T-2) 및 미세 분진 흡입 위험이 있으므로 바람 부는 날 경작지 주변 통과 시 호흡기 보호 주의.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>주차장 (인공 포장 대조구)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Paved Parking Lot Control</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>인공 포장면 (음성 대조군)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>관리사무소 앞 아스팔트 포장면, 식생 완전 부재</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>7</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>363.9</v>
+      </c>
+      <c r="I6" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>4월 (456 CFU/㎥), 7월 (326 CFU/㎥)</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>326</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>미포집 (하절기 집중 관측)</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Fusarium (33.4%), Coprinellus radians (29.8%), Nectriaceae (18.3%), Penicillium (13.4%)</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>연중 평균 363.9 CFU/㎥로 10개 지점 중 최저치. 전 조사 기간 동안 환경부 실내 권고기준(500 CFU/㎥)을 상시 만족하는 유일한 지점.</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>수목 및 낙엽층 부재 시 자연계 진균 포자 방출원이 형성되지 않음을 역설적으로 입증하는 '음성 대조군(Negative Control)'. 관측 균주는 주로 인근 도로/차량 비산 먼지 유래.</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>진균 포자는 적으나 아스팔트 복사열 및 차량 배기가스가 존재하므로 산림 치유 목적으로 머무르는 공간은 아님.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>소나무림</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Pinus densiflora Siebold &amp; Zucc.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>온대 천연 침엽수림</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>중턱 능선 사면 온대 자연림, 풍부한 간벌 고사목</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="G7" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="H7" t="n">
+        <v>539</v>
+      </c>
+      <c r="I7" t="n">
+        <v>172.3</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>7월 (750 CFU/㎥), 8월 (746 CFU/㎥)</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>750</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Capnodiales (28.2%), Penicillium (17.5%), Cladosporium (16.3%), Umbelopsis (16.2%)</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Coprinellus radians (59.4% 절대 우점), Irpex laceratus (11.8%), Capnodiales (9.6%), Trichoderma (8.9%)</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>여름철 담자균문 백색부후균 Coprinellus radians(방사형먹물버섯류, 59.4%)와 Irpex laceratus(11.8%)가 71.2%를 합작 독점.</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>소나무 고사목과 간벌재 리그닌을 분해하여 난분해성 유기물을 토양 부식토로 전환시키는 탄소 순환의 핵심 현장. 자연 임분의 성숙도와 목재 부후 과정의 핵심 지표.</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>미세 담자포자(2~4㎛)가 비산하므로 버섯 포자 알레르기 유증상자는 강우 직후 방문 시 마스크 착용 권장. 평상시 소나무 피톤치드 효과 우수.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>일본잎갈나무림 a (낙엽송 a)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Larix kaempferi (Stand A)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>낙엽성 침엽수 인공림</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>남동사면 완경사지, 일조 투과 및 통풍 우수</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="G8" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="H8" t="n">
+        <v>444.3</v>
+      </c>
+      <c r="I8" t="n">
+        <v>34</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>5월 초여름 (868 CFU/㎥), 7월 (640 CFU/㎥)</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>640</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Capnodiales (63.7%), Alternaria (13.7%), Cladosporium (11.1%)</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Cladosporium (24.4%), Capnodiales (23.2%), Trichoderma (22.8%), Penicillium (12.2%), Fusarium (10.8%)</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>연중 평균 444 CFU/㎥로 전체 산림 임분 중 가장 청정. 특정 종의 독점 없이 Capnodiales, Cladosporium, Trichoderma가 균형을 이룸.</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>낙엽송 특유의 광 투과성과 우수한 공기 유동성으로 인해 임내 습도 정체가 발생하지 않음. 안정적 낙엽 분해와 청정한 수관 환경 형성.</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>대기질이 가장 청정하고 피톤치드가 안정적으로 발산되어 **학술림 내 최적의 산림 치유 산책 코스로 적극 추천**.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>버들나무림 b (왕버들 b)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Salix koreensis (Stand B)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>수변 계곡 하류 활엽수림</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>계곡 하류 퇴적지, 고수위 및 퇴적 유기물 풍부</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="G9" t="n">
+        <v>40.8</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1214</v>
+      </c>
+      <c r="I9" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>4월 봄철 (1,658 CFU/㎥, 봄철 전 지점 1위)</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>1298</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Capnodiales (71.0%), Alternaria (13.0%), Eukaryota (7.1%), Coprinellus (3.3%)</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Trichoderma (29.7%), Fusarium (27.0%), Colletotrichum gloeosporioides (24.2%), Alternaria (4.5%)</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>봄철 신엽 개엽기 Cladosporium/Capnodiales 조기 대량 비산(1,658) 및 여름철 활엽수 탄저병균 Colletotrichum(24.2%)의 집중 발생.</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>계곡 상류로부터 운반된 유기물 집적과 높은 습도로 인해 수변 미생물 대사 활성이 극대화됨. 왕버들 탄저병 발생 모니터링의 핵심 지표.</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>4월에 1급 알레르겐 포자 농도가 높으므로 알레르기 비염 및 천식 환자는 봄철 진입 시 주의 필요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>일본잎갈나무림 b (낙엽송 b)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Larix kaempferi (Stand B)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>경사지 낙엽송 임분</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>사면 상단부 능선 바람받이 사면</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>6</v>
+      </c>
+      <c r="G10" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="H10" t="n">
+        <v>930</v>
+      </c>
+      <c r="I10" t="n">
+        <v>357.7</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>4월 봄철 (1,146 CFU/㎥, 세균 1,954 CFU/㎥)</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>472</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Capnodiales (49.2%), Fusarium (24.6%), Clonostachys (11.2%), Alternaria (9.5%)</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Aspergillus (30.9%), Fusarium (25.4%), Trichoderma (17.4%), Ceriporia lacerata (9.5%)</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>4월 건조 강풍(최대 16.3m/s) 시 엽면 피생균(Capnodiales 49%) 및 토양 세균(1,954)의 일시적 풍식 비산. 여름철 목재부후균 Ceriporia(9.5%) 출현.</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>바람받이 사면의 물리적 미기후 역학을 반영하며, 계절 간 기상 변동에 민감하게 반응하는 산림 대기 완충 지표 임분.</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>봄철 강풍 시 일시적으로 미세 입자 비산이 많으므로 방풍 안경 및 마스크 착용이 유리함.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>잣나무림 b</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Pinus koraiensis (Stand B)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>능선 연접 잣나무림</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>상부 능선부 연접 사면, 통풍 양호</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="G11" t="n">
+        <v>33.4</v>
+      </c>
+      <c r="H11" t="n">
+        <v>520.7</v>
+      </c>
+      <c r="I11" t="n">
+        <v>23.7</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>8월 늦여름 (912 CFU/㎥), 7월 (638 CFU/㎥)</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>638</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Penicillium mallochii (50.1%), Capnodiales (32.1%), Coprinellus (15.1%)</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Trichoderma (80.2%), Aspergillus (9.7%), Bjerkandera (8.5%), Oudemansiella (1.1%)</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>봄철 Penicillium mallochii(50.1%) 우점에서 여름철 Trichoderma(80.2%)로의 전환. 계곡부 Stand A 대비 진균 농도가 절반 이하로 안정적 억제.</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>동일 잣나무 수종임에도 능선 지형의 우수한 통풍성으로 인해 습도 정체가 해소되어 진균 농도가 크게 낮아짐. '지형 미기후 조절 메커니즘'의 증거.</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>잣나무 피톤치드 치유 효과를 누리면서도 고습도 곰팡이 포자를 회피할 수 있는 최적의 힐링 코스.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>